<commit_message>
Rebuild financial model to final structure (SBA $450K + bank $300K + equity $195K)
- model.py: SBA $450K/15yr/10.5% (startup+WC only); acquisition financed by a
  concurrent $300K/6%/3yr bank term loan (LICENSE_PAID_AT_CLOSE=False); equity $195K
- Regenerated all three workbooks
- Authoritative: sources $945K; DSCR 1.79x/4.02x/5.95x (global 3.92x); min cash $444,962
- Record locked decisions + stress/piggyback caveats in COUNSEL_QA_REVIEW

https://claude.ai/code/session_01GAHLyfqLR9bxwN2jm6VjPU
</commit_message>
<xml_diff>
--- a/financial_models/output/Azalea_Hospice_Investor_Package.xlsx
+++ b/financial_models/output/Azalea_Hospice_Investor_Package.xlsx
@@ -1215,22 +1215,22 @@
     </comment>
     <comment ref="B110" authorId="0" shapeId="0">
       <text>
-        <t>Sized to pay the seller in full at close + fund startup costs and working-capital reserve. FLAG / CONFIRM: go-forward assumption, not in Paloma actuals.</t>
+        <t>Sized for startup costs + working-capital reserve (the Hickory acquisition is funded by the bank term loan below). FLAG / CONFIRM: go-forward assumption, not in Paloma actuals.</t>
       </text>
     </comment>
     <comment ref="B111" authorId="0" shapeId="0">
       <text>
-        <t>FLAG / CONFIRM: go-forward assumption, not in Paloma actuals.</t>
+        <t>Typical 7(a) variable: Prime ~7.5% + 3.0% spread. FLAG / CONFIRM: go-forward assumption, not in Paloma actuals.</t>
       </text>
     </comment>
     <comment ref="B112" authorId="0" shapeId="0">
       <text>
-        <t>10-year amortization. FLAG / CONFIRM: go-forward assumption, not in Paloma actuals.</t>
+        <t>15-year amortization. FLAG / CONFIRM: go-forward assumption, not in Paloma actuals.</t>
       </text>
     </comment>
     <comment ref="B113" authorId="0" shapeId="0">
       <text>
-        <t>Cash capital contribution by James Bullard (19.5% passive member). FLAG / CONFIRM: go-forward assumption, not in Paloma actuals.</t>
+        <t>Cash capital contribution by James Bullard (19.5% passive member); $180K designated as the SBA equity injection. FLAG / CONFIRM: go-forward assumption, not in Paloma actuals.</t>
       </text>
     </comment>
     <comment ref="B114" authorId="0" shapeId="0">
@@ -1265,22 +1265,22 @@
     </comment>
     <comment ref="B120" authorId="0" shapeId="0">
       <text>
-        <t>CHOW: acquire Hickory Hospice's existing Medicare-certified provider number (San Antonio + Tyler alternative-delivery site). Eliminates 855A enrollment gap - Azalea bills from day 1.</t>
+        <t>CHOW: purchase 100% of Hickory Hospice LLC's membership interests; its Medicare-certified provider number conveys with the entity (Azalea bills from day 1). Funded by the bank term loan below.</t>
       </text>
     </comment>
     <comment ref="B121" authorId="0" shapeId="0">
       <text>
-        <t>Seller financing on the license acquisition.</t>
+        <t>Concurrent bank term loan (Jim Bullard's bank); Jim personally guarantees. Subordinate to the SBA loan.</t>
       </text>
     </comment>
     <comment ref="B122" authorId="0" shapeId="0">
       <text>
-        <t>Monthly P+I amortization.</t>
+        <t>3-year monthly P+I amortization.</t>
       </text>
     </comment>
     <comment ref="B123" authorId="0" shapeId="0">
       <text>
-        <t>GAAP intangible amortization - non-cash, below EBITDA. No effect on DSCR.</t>
+        <t>GAAP intangible amortization - non-cash, below EBITDA. No effect on DSCR. Confirm tax treatment of a membership-interest purchase with CPA.</t>
       </text>
     </comment>
     <comment ref="B126" authorId="0" shapeId="0">
@@ -3424,7 +3424,7 @@
         </is>
       </c>
       <c r="B110" s="9" t="n">
-        <v>555000</v>
+        <v>450000</v>
       </c>
     </row>
     <row r="111">
@@ -3434,7 +3434,7 @@
         </is>
       </c>
       <c r="B111" s="7" t="n">
-        <v>0.115</v>
+        <v>0.105</v>
       </c>
     </row>
     <row r="112">
@@ -3444,7 +3444,7 @@
         </is>
       </c>
       <c r="B112" s="17" t="n">
-        <v>120</v>
+        <v>180</v>
       </c>
     </row>
     <row r="113">
@@ -3520,7 +3520,7 @@
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>Hickory Medicare license - acquisition cost ($)</t>
+          <t>Hickory acquisition - purchase price ($)</t>
         </is>
       </c>
       <c r="B120" s="9" t="n">
@@ -3530,7 +3530,7 @@
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>License note interest rate (APR)</t>
+          <t>Acquisition bank loan rate (APR)</t>
         </is>
       </c>
       <c r="B121" s="7" t="n">
@@ -3540,7 +3540,7 @@
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>License note term (months)</t>
+          <t>Acquisition bank loan term (months)</t>
         </is>
       </c>
       <c r="B122" s="17" t="n">
@@ -3550,7 +3550,7 @@
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>License intangible amortization life (yrs)</t>
+          <t>Acquisition intangible amortization life (yrs)</t>
         </is>
       </c>
       <c r="B123" s="17" t="n">
@@ -3672,11 +3672,11 @@
     <row r="139">
       <c r="A139" s="12" t="inlineStr">
         <is>
-          <t>Opening cash = equity + loan - startup - capex - license (paid at close)</t>
+          <t>Opening cash = equity + loan - startup - capex</t>
         </is>
       </c>
       <c r="B139" s="23">
-        <f>Inputs!$B$113+Inputs!$B$110-Inputs!$B$138-Inputs!$B$117-Inputs!$B$120</f>
+        <f>Inputs!$B$113+Inputs!$B$110-Inputs!$B$138-Inputs!$B$117</f>
         <v/>
       </c>
     </row>
@@ -7422,7 +7422,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Debt Schedule - SBA 7(a) only (seller paid at close) | DSCR shown (target &gt;= 1.25x)</t>
+          <t>Debt Schedule - SBA 7(a) + Hickory license seller note | Combined DSCR shown (target &gt;= 1.25x)</t>
         </is>
       </c>
     </row>
@@ -7451,7 +7451,7 @@
         </is>
       </c>
       <c r="B6" s="24">
-        <f>0</f>
+        <f>PMT(Inputs!$B$121/12,Inputs!$B$122,-Inputs!$B$120)</f>
         <v/>
       </c>
     </row>
@@ -8025,7 +8025,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>HICKORY LICENSE - PAID AT CLOSE (no seller note; schedule zeroed)</t>
+          <t>HICKORY LICENSE SELLER NOTE ($300K, 6%, 36 mo)</t>
         </is>
       </c>
     </row>
@@ -8036,7 +8036,7 @@
         </is>
       </c>
       <c r="C18" s="26">
-        <f>0</f>
+        <f>Inputs!$B$120</f>
         <v/>
       </c>
       <c r="D18" s="24">
@@ -8467,7 +8467,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>DEBT SERVICE &amp; COVERAGE (SBA only)</t>
+          <t>COMBINED DEBT SERVICE &amp; COVERAGE</t>
         </is>
       </c>
     </row>
@@ -8648,7 +8648,7 @@
     <row r="27">
       <c r="A27" s="28" t="inlineStr">
         <is>
-          <t>TOTAL DEBT SERVICE (P+I)</t>
+          <t>TOTAL DEBT SERVICE (P+I, combined)</t>
         </is>
       </c>
       <c r="C27" s="23">
@@ -8822,7 +8822,7 @@
     <row r="29">
       <c r="A29" s="28" t="inlineStr">
         <is>
-          <t>DSCR (period)</t>
+          <t>COMBINED DSCR (period)</t>
         </is>
       </c>
       <c r="C29" s="58">
@@ -11265,7 +11265,7 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>0</f>
+        <f>Inputs!$B$120</f>
         <v/>
       </c>
       <c r="C34" s="26">

</xml_diff>